<commit_message>
Made presentation and added footprintst
I finished the presentation. This required me to remove some things from the simulation to make it more understandable. I also just about finished adding all the footprints for the PCB
</commit_message>
<xml_diff>
--- a/Battery Charger Project/Docs/Data sheets/Gen data.xlsx
+++ b/Battery Charger Project/Docs/Data sheets/Gen data.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Verrazano\Acedemic\Research\Battery Charger Project\Data sheets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Verrazano\Acedemic\Research\Battery-Charger\Battery Charger Project\Docs\Data sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A624D45-733F-4390-A6D8-89806F4C288F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F322EFB0-10F7-44F1-8DD3-AAF1D9BF4216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{122414F2-41E6-48D7-A7EA-B912A1A3DDA8}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{122414F2-41E6-48D7-A7EA-B912A1A3DDA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -213,15 +213,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>V</a:t>
-            </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="-25000"/>
-              <a:t>LL_p </a:t>
+              <a:t>Generator</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t>vs Shaft RPM</a:t>
+              <a:t> Output</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -260,18 +256,18 @@
     <c:plotArea>
       <c:layout/>
       <c:scatterChart>
-        <c:scatterStyle val="smoothMarker"/>
+        <c:scatterStyle val="lineMarker"/>
         <c:varyColors val="0"/>
         <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
+          <c:idx val="0"/>
+          <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$F$2</c:f>
+              <c:f>Sheet1!$G$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>VLL_p</c:v>
+                  <c:v>hz</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -279,71 +275,83 @@
           <c:spPr>
             <a:ln w="19050" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent2"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="none"/>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$D$3:$D$19</c:f>
+              <c:f>Sheet1!$G$3:$G$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="17"/>
                 <c:pt idx="0">
-                  <c:v>68</c:v>
+                  <c:v>7.31</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>116</c:v>
+                  <c:v>11.75</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>166</c:v>
+                  <c:v>16.670000000000002</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>217</c:v>
+                  <c:v>21.75</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>268</c:v>
+                  <c:v>29.96</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>333</c:v>
+                  <c:v>33.299999999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>388</c:v>
+                  <c:v>38.75</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>440</c:v>
+                  <c:v>43.99</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>490</c:v>
+                  <c:v>48.99</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>545</c:v>
+                  <c:v>54.36</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>597</c:v>
+                  <c:v>59.8</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>653</c:v>
+                  <c:v>65.260000000000005</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>705</c:v>
+                  <c:v>70.569999999999993</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>753</c:v>
+                  <c:v>75.150000000000006</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>805</c:v>
+                  <c:v>80.489999999999995</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>858</c:v>
+                  <c:v>85.73</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>918</c:v>
+                  <c:v>92.01</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -408,14 +416,15 @@
               </c:numCache>
             </c:numRef>
           </c:yVal>
-          <c:smooth val="1"/>
+          <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-0015-4750-8AF8-5D2D3C5DF770}"/>
+              <c16:uniqueId val="{00000003-F4E0-446B-A0C5-294099B5AE50}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="t"/>
           <c:showLegendKey val="0"/>
           <c:showVal val="0"/>
           <c:showCatName val="0"/>
@@ -423,188 +432,11 @@
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
         </c:dLbls>
-        <c:axId val="463387615"/>
-        <c:axId val="463387199"/>
-        <c:extLst>
-          <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-            <c15:filteredScatterSeries>
-              <c15:ser>
-                <c:idx val="0"/>
-                <c:order val="0"/>
-                <c:tx>
-                  <c:strRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Sheet1!$E$2</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:strCache>
-                      <c:ptCount val="1"/>
-                      <c:pt idx="0">
-                        <c:v>VLL_rms</c:v>
-                      </c:pt>
-                    </c:strCache>
-                  </c:strRef>
-                </c:tx>
-                <c:spPr>
-                  <a:ln w="19050" cap="rnd">
-                    <a:solidFill>
-                      <a:schemeClr val="accent1"/>
-                    </a:solidFill>
-                    <a:round/>
-                  </a:ln>
-                  <a:effectLst/>
-                </c:spPr>
-                <c:marker>
-                  <c:symbol val="none"/>
-                </c:marker>
-                <c:xVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Sheet1!$D$3:$D$19</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="17"/>
-                      <c:pt idx="0">
-                        <c:v>68</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>116</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>166</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>217</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>268</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>333</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>388</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>440</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>490</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>545</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>597</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>653</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>705</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>753</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>805</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>858</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>918</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:xVal>
-                <c:yVal>
-                  <c:numRef>
-                    <c:extLst>
-                      <c:ext uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
-                        <c15:formulaRef>
-                          <c15:sqref>Sheet1!$E$3:$E$19</c15:sqref>
-                        </c15:formulaRef>
-                      </c:ext>
-                    </c:extLst>
-                    <c:numCache>
-                      <c:formatCode>General</c:formatCode>
-                      <c:ptCount val="17"/>
-                      <c:pt idx="0">
-                        <c:v>7.64</c:v>
-                      </c:pt>
-                      <c:pt idx="1">
-                        <c:v>12.9</c:v>
-                      </c:pt>
-                      <c:pt idx="2">
-                        <c:v>18.3</c:v>
-                      </c:pt>
-                      <c:pt idx="3">
-                        <c:v>24.3</c:v>
-                      </c:pt>
-                      <c:pt idx="4">
-                        <c:v>30.3</c:v>
-                      </c:pt>
-                      <c:pt idx="5">
-                        <c:v>37.299999999999997</c:v>
-                      </c:pt>
-                      <c:pt idx="6">
-                        <c:v>43.3</c:v>
-                      </c:pt>
-                      <c:pt idx="7">
-                        <c:v>48.9</c:v>
-                      </c:pt>
-                      <c:pt idx="8">
-                        <c:v>54.6</c:v>
-                      </c:pt>
-                      <c:pt idx="9">
-                        <c:v>60.4</c:v>
-                      </c:pt>
-                      <c:pt idx="10">
-                        <c:v>66.8</c:v>
-                      </c:pt>
-                      <c:pt idx="11">
-                        <c:v>72.7</c:v>
-                      </c:pt>
-                      <c:pt idx="12">
-                        <c:v>78.599999999999994</c:v>
-                      </c:pt>
-                      <c:pt idx="13">
-                        <c:v>83.8</c:v>
-                      </c:pt>
-                      <c:pt idx="14">
-                        <c:v>89.6</c:v>
-                      </c:pt>
-                      <c:pt idx="15">
-                        <c:v>95.3</c:v>
-                      </c:pt>
-                      <c:pt idx="16">
-                        <c:v>102</c:v>
-                      </c:pt>
-                    </c:numCache>
-                  </c:numRef>
-                </c:yVal>
-                <c:smooth val="1"/>
-                <c:extLst>
-                  <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                    <c16:uniqueId val="{00000000-0015-4750-8AF8-5D2D3C5DF770}"/>
-                  </c:ext>
-                </c:extLst>
-              </c15:ser>
-            </c15:filteredScatterSeries>
-          </c:ext>
-        </c:extLst>
+        <c:axId val="1770667856"/>
+        <c:axId val="1392202064"/>
       </c:scatterChart>
       <c:valAx>
-        <c:axId val="463387615"/>
+        <c:axId val="1770667856"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -624,20 +456,66 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
-        <c:minorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Shaft</a:t>
+                </a:r>
+                <a:r>
+                  <a:rPr lang="en-US" baseline="0"/>
+                  <a:t> Frequency (Hz)</a:t>
+                </a:r>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
           <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="5000"/>
-                  <a:lumOff val="95000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
             </a:ln>
             <a:effectLst/>
           </c:spPr>
-        </c:minorGridlines>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -675,12 +553,12 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="463387199"/>
+        <c:crossAx val="1392202064"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
       <c:valAx>
-        <c:axId val="463387199"/>
+        <c:axId val="1392202064"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -700,6 +578,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>VLL_p (V)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="0.0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -737,470 +670,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="463387615"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:legend>
-      <c:legendPos val="b"/>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:legend>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="bg1"/>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout/>
-      <c:scatterChart>
-        <c:scatterStyle val="lineMarker"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:spPr>
-            <a:ln w="19050" cap="rnd">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="circle"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:dispRSqr val="0"/>
-            <c:dispEq val="1"/>
-            <c:trendlineLbl>
-              <c:numFmt formatCode="General" sourceLinked="0"/>
-              <c:spPr>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-              <c:txPr>
-                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr>
-                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                      <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
-                      </a:solidFill>
-                      <a:latin typeface="+mn-lt"/>
-                      <a:ea typeface="+mn-ea"/>
-                      <a:cs typeface="+mn-cs"/>
-                    </a:defRPr>
-                  </a:pPr>
-                  <a:endParaRPr lang="en-US"/>
-                </a:p>
-              </c:txPr>
-            </c:trendlineLbl>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$3:$F$19</c:f>
-              <c:numCache>
-                <c:formatCode>0.0</c:formatCode>
-                <c:ptCount val="17"/>
-                <c:pt idx="0">
-                  <c:v>10.804591616530447</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>18.243354954612929</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>25.880108191427642</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>34.365389565666213</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>42.850670939904781</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>52.750165876516448</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>61.235447250755016</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>69.155043200044346</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>77.216060505570994</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>85.418499167334943</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>94.469465966522748</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>102.81332598452403</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>111.15718600252526</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>118.51109652686537</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>126.71353518862932</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>134.77455249415596</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>144.24978336205569</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$G$3:$G$19</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="17"/>
-                <c:pt idx="1">
-                  <c:v>11.75</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>16.670000000000002</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>21.75</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>29.96</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>33.299999999999997</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>38.75</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>43.99</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>48.99</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>54.36</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>59.8</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>65.260000000000005</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>70.569999999999993</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>75.150000000000006</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>80.489999999999995</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>85.73</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>92.01</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2908-440B-B383-62CC0BE4E4FC}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:axId val="1675556527"/>
-        <c:axId val="1675562767"/>
-      </c:scatterChart>
-      <c:valAx>
-        <c:axId val="1675556527"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="0.0" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1675562767"/>
-        <c:crosses val="autoZero"/>
-        <c:crossBetween val="midCat"/>
-      </c:valAx>
-      <c:valAx>
-        <c:axId val="1675562767"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="15000"/>
-                  <a:lumOff val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="nextTo"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-            <a:solidFill>
-              <a:schemeClr val="tx1">
-                <a:lumMod val="25000"/>
-                <a:lumOff val="75000"/>
-              </a:schemeClr>
-            </a:solidFill>
-            <a:round/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="tx1">
-                    <a:lumMod val="65000"/>
-                    <a:lumOff val="35000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="1675556527"/>
+        <c:crossAx val="1770667856"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1289,46 +759,6 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -1845,543 +1275,27 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="bg1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln>
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="1">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="15000"/>
-            <a:lumOff val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="5000"/>
-            <a:lumOff val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="35000"/>
-            <a:lumOff val="65000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="19050" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:prstDash val="sysDot"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:noFill/>
-      <a:ln>
-        <a:noFill/>
-      </a:ln>
-    </cs:spPr>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>251460</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>54429</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>65314</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>594360</xdr:colOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>359229</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:rowOff>32657</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="2" name="Chart 1">
+        <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF8A5436-8D4A-4D79-A8A6-48E2EB412B4C}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2404826-A698-DFA8-6468-30C34871979C}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2394,42 +1308,6 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>246529</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>533400</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>26894</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="4" name="Chart 3">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44EAF72F-30B4-9053-3CD3-382A96C4ED61}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2735,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4562E0B5-54E2-481D-808C-A42013EC5463}">
-  <dimension ref="A2:G23"/>
+  <dimension ref="A2:G19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="11.88671875" customWidth="1"/>
@@ -2788,7 +1666,9 @@
         <f>E3*SQRT(2)</f>
         <v>10.804591616530447</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2">
+        <v>7.31</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
@@ -3188,18 +2068,6 @@
       </c>
       <c r="G19" s="1">
         <v>92.01</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D23">
-        <v>25</v>
-      </c>
-      <c r="E23">
-        <v>48</v>
-      </c>
-      <c r="F23">
-        <f>E23*D23</f>
-        <v>1200</v>
       </c>
     </row>
   </sheetData>
@@ -3210,6 +2078,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100828C9112DD8F15449225F064D66EBDFE" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b81720e2d1e30b7fbbac34e4ce0795be">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="c971a386-8160-44b9-bb17-0adc33850141" xmlns:ns4="30c13f3f-6095-4dfb-a332-3c3ec0a6667d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ee2ef5a2c475d390c372d43812c0b725" ns3:_="" ns4:_="">
     <xsd:import namespace="c971a386-8160-44b9-bb17-0adc33850141"/>
@@ -3424,15 +2301,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -3440,6 +2308,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF203C4B-30FD-4C6C-B8C6-ADCEEC0734AC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7AC1DE57-DDF7-4F30-8FFA-8F3B9AD2559D}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3454,14 +2330,6 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EF203C4B-30FD-4C6C-B8C6-ADCEEC0734AC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>